<commit_message>
Mejorar gestion de stock en carrito y actualizar documentacion de entrega.
Descuenta y restaura stock al agregar, actualizar o eliminar del carrito; corrige Mercado Pago en local y anade guia demo, informes y tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Casos_Integracion_Ferramas.xlsx
+++ b/docs/Casos_Integracion_Ferramas.xlsx
@@ -2282,7 +2282,7 @@
       </c>
       <c r="C13" s="68" t="inlineStr">
         <is>
-          <t>Fitzroyal</t>
+          <t>Jose Larenas / Oscar Oviedo</t>
         </is>
       </c>
       <c r="D13" s="90" t="n"/>
@@ -2396,7 +2396,7 @@
       </c>
       <c r="D21" s="73" t="inlineStr">
         <is>
-          <t>Fitzroyal</t>
+          <t>Jose Larenas / Oscar Oviedo</t>
         </is>
       </c>
       <c r="E21" s="94" t="n"/>

</xml_diff>